<commit_message>
Xử lý số 0
</commit_message>
<xml_diff>
--- a/convert/Bao cao vi pham.xlsx
+++ b/convert/Bao cao vi pham.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18688" uniqueCount="1838">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18681" uniqueCount="1838">
   <si>
     <t>2022-03-01</t>
   </si>
@@ -10363,8 +10363,8 @@
       <c r="AC61">
         <v>25</v>
       </c>
-      <c r="AE61" t="s">
-        <v>37</v>
+      <c r="AE61">
+        <v>240</v>
       </c>
       <c r="AG61">
         <v>12</v>
@@ -15302,8 +15302,8 @@
       <c r="U117" t="s">
         <v>36</v>
       </c>
-      <c r="AE117" t="s">
-        <v>37</v>
+      <c r="AE117">
+        <v>240</v>
       </c>
       <c r="AG117">
         <v>114</v>
@@ -36098,8 +36098,8 @@
       <c r="E345" t="s">
         <v>908</v>
       </c>
-      <c r="AE345" t="s">
-        <v>37</v>
+      <c r="AE345">
+        <v>240</v>
       </c>
       <c r="AO345" t="s">
         <v>36</v>
@@ -40594,8 +40594,8 @@
       <c r="W394" t="s">
         <v>36</v>
       </c>
-      <c r="AE394" t="s">
-        <v>37</v>
+      <c r="AE394">
+        <v>240</v>
       </c>
       <c r="AP394">
         <v>240</v>
@@ -41473,8 +41473,8 @@
       <c r="E406" t="s">
         <v>1078</v>
       </c>
-      <c r="AE406" t="s">
-        <v>37</v>
+      <c r="AE406">
+        <v>240</v>
       </c>
     </row>
     <row r="407" spans="1:68">
@@ -42027,8 +42027,8 @@
       <c r="T413">
         <v>1</v>
       </c>
-      <c r="AE413" t="s">
-        <v>37</v>
+      <c r="AE413">
+        <v>240</v>
       </c>
       <c r="AP413">
         <v>1</v>
@@ -50328,8 +50328,8 @@
       <c r="R503">
         <v>1</v>
       </c>
-      <c r="AE503" t="s">
-        <v>37</v>
+      <c r="AE503">
+        <v>240</v>
       </c>
     </row>
     <row r="504" spans="1:68">

</xml_diff>